<commit_message>
report for condition based maintenance added
</commit_message>
<xml_diff>
--- a/results/pulp_same_case_results.xlsx
+++ b/results/pulp_same_case_results.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Schedule" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Bottleneck" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Condition Maintenance" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,10 +482,10 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="G2" t="n">
-        <v>0.47</v>
+        <v>0.213</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -1218,4 +1219,730 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>solver</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>daily_usage_min</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>threshold_min</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>maintenance_required</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>maintenance_reserved_min</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>112</v>
+      </c>
+      <c r="E2" t="n">
+        <v>180</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>180</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>180</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>180</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>180</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>96</v>
+      </c>
+      <c r="E7" t="n">
+        <v>180</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>180</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>180</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>180</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>180</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>48</v>
+      </c>
+      <c r="E12" t="n">
+        <v>180</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>180</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>180</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>180</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>180</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>84</v>
+      </c>
+      <c r="E17" t="n">
+        <v>180</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>180</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>180</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>180</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>180</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>140</v>
+      </c>
+      <c r="E22" t="n">
+        <v>180</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>180</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>180</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>180</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>180</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
condtioned changed so that the threshhold get clicked for pulp and pyomo case + report also changed based on this
</commit_message>
<xml_diff>
--- a/results/pulp_same_case_results.xlsx
+++ b/results/pulp_same_case_results.xlsx
@@ -8,9 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Schedule" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Bottleneck" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Condition Maintenance" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Schedule_same_case" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Bottleneck_same_case" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Condition_same_case" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Schedule_maint_stress" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Bottleneck_maint_stress" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Condition_maint_stress" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,46 +419,86 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="35" customWidth="1" min="13" max="13"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>solver</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>orders</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>operations</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>makespan_min</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>total_tardiness_min</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>maintenance_triggers</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>reserved_maintenance_min</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>max_daily_usage_min</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>binary_variables</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>solve_time_sec</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>formulation</t>
         </is>
@@ -464,30 +507,96 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" t="n">
         <v>12</v>
       </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>168</v>
       </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>140</v>
+      </c>
+      <c r="K2" t="n">
         <v>116</v>
       </c>
-      <c r="G2" t="n">
-        <v>0.213</v>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="L2" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>MILP with big-M and binary ordering variables</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F3" t="n">
+        <v>680</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" t="n">
+        <v>180</v>
+      </c>
+      <c r="J3" t="n">
+        <v>376</v>
+      </c>
+      <c r="K3" t="n">
+        <v>116</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>MILP with big-M and binary ordering variables</t>
         </is>
@@ -504,579 +613,658 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>operation_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>order_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>batch_id</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>product_id</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>machine</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>duration</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>start_min</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>end_min</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>start_day</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>end_day</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>3</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>O2</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>O2_B1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Cutting</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>8</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>32</v>
       </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
       <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
         <v>32</v>
       </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
       <c r="K2" t="n">
         <v>1</v>
       </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>9</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>O4</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>O4_B1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Drilling</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>12</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>48</v>
       </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
       <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
         <v>48</v>
       </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
       <c r="K3" t="n">
         <v>1</v>
       </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>8</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>O3</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>O3_B1</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Painting</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>6</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>24</v>
       </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
       <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
         <v>24</v>
       </c>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
       <c r="K4" t="n">
         <v>1</v>
       </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>5</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>O2</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>O2_B1</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Painting</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>8</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>40</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>32</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>72</v>
       </c>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
       <c r="K5" t="n">
         <v>1</v>
       </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>0</v>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>O1</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>O1_B1</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Cutting</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>10</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>50</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>35</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>85</v>
       </c>
-      <c r="J6" t="n">
-        <v>1</v>
-      </c>
       <c r="K6" t="n">
         <v>1</v>
       </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>7</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>O3</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>O3_B1</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Drilling</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>6</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>18</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>48</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>66</v>
       </c>
-      <c r="J7" t="n">
-        <v>1</v>
-      </c>
       <c r="K7" t="n">
         <v>1</v>
       </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>10</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>O4</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>O4_B1</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Welding</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>12</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>84</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>48</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>132</v>
       </c>
-      <c r="J8" t="n">
-        <v>1</v>
-      </c>
       <c r="K8" t="n">
         <v>1</v>
       </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>4</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>O2</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>O2_B1</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Milling</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>8</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>48</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>72</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>120</v>
       </c>
-      <c r="J9" t="n">
-        <v>1</v>
-      </c>
       <c r="K9" t="n">
         <v>1</v>
       </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>2</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>O1</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>O1_B1</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Painting</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>10</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>40</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>85</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>125</v>
       </c>
-      <c r="J10" t="n">
-        <v>1</v>
-      </c>
       <c r="K10" t="n">
         <v>1</v>
       </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>6</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>O3</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>O3_B1</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Cutting</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>6</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>30</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>90</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>120</v>
       </c>
-      <c r="J11" t="n">
-        <v>1</v>
-      </c>
       <c r="K11" t="n">
         <v>1</v>
       </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>O4</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>O4_B1</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Painting</t>
         </is>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>12</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>36</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>132</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>168</v>
       </c>
-      <c r="J12" t="n">
-        <v>1</v>
-      </c>
       <c r="K12" t="n">
         <v>1</v>
       </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>O1</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>O1_B1</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Drilling</t>
         </is>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>10</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>30</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>138</v>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>168</v>
       </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
       <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1091,8 +1279,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1120,6 +1316,11 @@
           <t>bottleneck_rank</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1139,6 +1340,11 @@
       <c r="E2" t="n">
         <v>1</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1158,6 +1364,11 @@
       <c r="E3" t="n">
         <v>2</v>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1177,6 +1388,11 @@
       <c r="E4" t="n">
         <v>3</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1196,6 +1412,11 @@
       <c r="E5" t="n">
         <v>4</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1214,6 +1435,11 @@
       </c>
       <c r="E6" t="n">
         <v>5</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>same_case</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1227,41 +1453,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>solver</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>machine</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>daily_usage_min</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>threshold_min</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>maintenance_required</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>maintenance_reserved_min</t>
         </is>
@@ -1270,675 +1511,2506 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Cutting</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
       <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
         <v>112</v>
       </c>
-      <c r="E2" t="n">
-        <v>180</v>
-      </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Cutting</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>2</v>
       </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
       <c r="E3" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Cutting</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>3</v>
       </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
       <c r="E4" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Cutting</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>4</v>
       </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
       <c r="E5" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>Cutting</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>5</v>
       </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
       <c r="E6" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>Drilling</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
       <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
         <v>96</v>
       </c>
-      <c r="E7" t="n">
-        <v>180</v>
-      </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Drilling</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>2</v>
       </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
       <c r="E8" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>Drilling</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>3</v>
       </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
       <c r="E9" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>Drilling</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>4</v>
       </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
       <c r="E10" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>Drilling</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>5</v>
       </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
       <c r="E11" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>Milling</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>1</v>
-      </c>
       <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
         <v>48</v>
       </c>
-      <c r="E12" t="n">
-        <v>180</v>
-      </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>Milling</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="D13" t="n">
         <v>2</v>
       </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
       <c r="E13" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>Milling</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="D14" t="n">
         <v>3</v>
       </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
       <c r="E14" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>Milling</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="D15" t="n">
         <v>4</v>
       </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
       <c r="E15" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>Milling</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="D16" t="n">
         <v>5</v>
       </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
       <c r="E16" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>Welding</t>
         </is>
       </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
       <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
         <v>84</v>
       </c>
-      <c r="E17" t="n">
-        <v>180</v>
-      </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>Welding</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="D18" t="n">
         <v>2</v>
       </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
       <c r="E18" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>Welding</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="D19" t="n">
         <v>3</v>
       </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
       <c r="E19" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>Welding</t>
         </is>
       </c>
-      <c r="C20" t="n">
+      <c r="D20" t="n">
         <v>4</v>
       </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
       <c r="E20" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>Welding</t>
         </is>
       </c>
-      <c r="C21" t="n">
+      <c r="D21" t="n">
         <v>5</v>
       </c>
-      <c r="D21" t="n">
-        <v>0</v>
-      </c>
       <c r="E21" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>Painting</t>
         </is>
       </c>
-      <c r="C22" t="n">
-        <v>1</v>
-      </c>
       <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
         <v>140</v>
       </c>
-      <c r="E22" t="n">
-        <v>180</v>
-      </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
           <t>Painting</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="D23" t="n">
         <v>2</v>
       </c>
-      <c r="D23" t="n">
-        <v>0</v>
-      </c>
       <c r="E23" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>Painting</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="D24" t="n">
         <v>3</v>
       </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
       <c r="E24" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
           <t>Painting</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="D25" t="n">
         <v>4</v>
       </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
       <c r="E25" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PuLP CBC</t>
+          <t>same_case</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
           <t>Painting</t>
         </is>
       </c>
-      <c r="C26" t="n">
+      <c r="D26" t="n">
         <v>5</v>
       </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>180</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>operation_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>batch_id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>product_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>duration</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>start_min</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>end_min</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>start_day</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>end_day</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>S4_B1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>32</v>
+      </c>
+      <c r="H2" t="n">
+        <v>96</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>96</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>S3_B1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>30</v>
+      </c>
+      <c r="H3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J3" t="n">
+        <v>180</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>S2_B1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>35</v>
+      </c>
+      <c r="H4" t="n">
+        <v>210</v>
+      </c>
+      <c r="I4" t="n">
+        <v>130</v>
+      </c>
+      <c r="J4" t="n">
+        <v>340</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>S1_B1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H5" t="n">
+        <v>160</v>
+      </c>
+      <c r="I5" t="n">
+        <v>140</v>
+      </c>
+      <c r="J5" t="n">
+        <v>300</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>S3_B1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H6" t="n">
+        <v>150</v>
+      </c>
+      <c r="I6" t="n">
+        <v>180</v>
+      </c>
+      <c r="J6" t="n">
+        <v>330</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>S4_B1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>32</v>
+      </c>
+      <c r="H7" t="n">
+        <v>224</v>
+      </c>
+      <c r="I7" t="n">
+        <v>256</v>
+      </c>
+      <c r="J7" t="n">
+        <v>480</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>S2_B1</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>35</v>
+      </c>
+      <c r="H8" t="n">
+        <v>140</v>
+      </c>
+      <c r="I8" t="n">
+        <v>340</v>
+      </c>
+      <c r="J8" t="n">
+        <v>480</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>S1_B1</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>40</v>
+      </c>
+      <c r="H9" t="n">
+        <v>120</v>
+      </c>
+      <c r="I9" t="n">
+        <v>360</v>
+      </c>
+      <c r="J9" t="n">
+        <v>480</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>S3_B1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>30</v>
+      </c>
+      <c r="H10" t="n">
+        <v>120</v>
+      </c>
+      <c r="I10" t="n">
+        <v>360</v>
+      </c>
+      <c r="J10" t="n">
+        <v>480</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>S1_B1</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>40</v>
+      </c>
+      <c r="H11" t="n">
+        <v>200</v>
+      </c>
+      <c r="I11" t="n">
+        <v>480</v>
+      </c>
+      <c r="J11" t="n">
+        <v>680</v>
+      </c>
+      <c r="K11" t="n">
+        <v>2</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>9</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>S4_B1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>32</v>
+      </c>
+      <c r="H12" t="n">
+        <v>128</v>
+      </c>
+      <c r="I12" t="n">
+        <v>480</v>
+      </c>
+      <c r="J12" t="n">
+        <v>608</v>
+      </c>
+      <c r="K12" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>S2_B1</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>35</v>
+      </c>
+      <c r="H13" t="n">
+        <v>175</v>
+      </c>
+      <c r="I13" t="n">
+        <v>505</v>
+      </c>
+      <c r="J13" t="n">
+        <v>680</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>machine_load_min</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>makespan_min</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>utilization_percent</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>bottleneck_rank</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>551</v>
+      </c>
+      <c r="C2" t="n">
+        <v>680</v>
+      </c>
+      <c r="D2" t="n">
+        <v>81.03</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>490</v>
+      </c>
+      <c r="C3" t="n">
+        <v>680</v>
+      </c>
+      <c r="D3" t="n">
+        <v>72.06</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>338</v>
+      </c>
+      <c r="C4" t="n">
+        <v>680</v>
+      </c>
+      <c r="D4" t="n">
+        <v>49.71</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>224</v>
+      </c>
+      <c r="C5" t="n">
+        <v>680</v>
+      </c>
+      <c r="D5" t="n">
+        <v>32.94</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>210</v>
+      </c>
+      <c r="C6" t="n">
+        <v>680</v>
+      </c>
+      <c r="D6" t="n">
+        <v>30.88</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>solver</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>daily_usage_min</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>threshold_min</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>maintenance_required</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>maintenance_reserved_min</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>290</v>
+      </c>
+      <c r="F2" t="n">
+        <v>180</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>200</v>
+      </c>
+      <c r="F3" t="n">
+        <v>180</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>180</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>180</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Cutting</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>180</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>210</v>
+      </c>
+      <c r="F7" t="n">
+        <v>180</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>128</v>
+      </c>
+      <c r="F8" t="n">
+        <v>180</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>180</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>180</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>180</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>210</v>
+      </c>
+      <c r="F12" t="n">
+        <v>180</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>180</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>180</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>180</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Milling</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>180</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>224</v>
+      </c>
+      <c r="F17" t="n">
+        <v>180</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>180</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>180</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>180</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Welding</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>180</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>376</v>
+      </c>
+      <c r="F22" t="n">
+        <v>180</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="n">
+        <v>175</v>
+      </c>
+      <c r="F23" t="n">
+        <v>180</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>180</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>180</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>maintenance_stress_case</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PuLP CBC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E26" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>